<commit_message>
Updated DZA_grids model - 2025-09-19 23:35
</commit_message>
<xml_diff>
--- a/VerveStacks_DZA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_DZA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DZA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{46E00F2E-B61A-4193-BD80-1BA039248023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2E379CE-7DA8-4ECE-AE3E-B1B9D0AAEBC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9311,7 +9311,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55CEA623-08FD-4B2F-A11D-AAA24F7E062B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A231929-6264-46A6-A287-93F16E2BE2D6}">
   <dimension ref="B9:D432"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -13979,7 +13979,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FC3E3D9-4A62-4D15-A8FA-A46920D69A30}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BDD7E4D-8607-4DBF-98EA-8120867E4AC1}">
   <dimension ref="B9:H432"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated DZA_grids model - 2025-09-20 09:06
</commit_message>
<xml_diff>
--- a/VerveStacks_DZA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_DZA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DZA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2E379CE-7DA8-4ECE-AE3E-B1B9D0AAEBC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C4A0C870-0ECF-4A00-A0F0-E3B1A8EE807A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9311,7 +9311,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A231929-6264-46A6-A287-93F16E2BE2D6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41A1A8CE-CED7-44D1-8BE3-F90C6E27F63D}">
   <dimension ref="B9:D432"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -13979,7 +13979,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BDD7E4D-8607-4DBF-98EA-8120867E4AC1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F79800D1-A76C-48B4-A0F8-14DC4D138B78}">
   <dimension ref="B9:H432"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated DZA_grids model - 2025-09-21 18:00
</commit_message>
<xml_diff>
--- a/VerveStacks_DZA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_DZA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DZA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97A57AB4-7163-476D-ADC6-8C5C0CA2890D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{92AC6249-1854-41FC-A412-C4278348FB5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8600,7 +8600,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62912341-A22D-4A6F-B101-7512428FE596}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C03E3B8D-F76F-40C0-B749-B78CCFA664A4}">
   <dimension ref="B9:D198"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10694,7 +10694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{056FC536-DB75-49C6-8C04-A87B8169AA72}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8C48D4C-4747-4328-BF13-1698AF82B930}">
   <dimension ref="B9:H198"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>